<commit_message>
fix BVA order payment test cases
</commit_message>
<xml_diff>
--- a/docs/testing/BVA/order & payment/Testcase_BVA_Order_Payment.xlsx
+++ b/docs/testing/BVA/order & payment/Testcase_BVA_Order_Payment.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="15732" windowHeight="8400"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="BVA_TestCases" sheetId="1" r:id="rId1"/>
@@ -30,30 +30,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="68">
   <si>
     <t>Test Case ID</t>
   </si>
   <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Mô tả tóm tắt</t>
-  </si>
-  <si>
-    <t>Trường test / Điểm biên BVA</t>
-  </si>
-  <si>
-    <t>Method</t>
-  </si>
-  <si>
-    <t>Endpoint</t>
-  </si>
-  <si>
-    <t>Inputs (Test Data / Request)</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
+    <t>Test summary / Description</t>
+  </si>
+  <si>
+    <t>Pre-condition</t>
+  </si>
+  <si>
+    <t>Test steps</t>
+  </si>
+  <si>
+    <t>Inputs (test data)</t>
+  </si>
+  <si>
+    <t>Expected result</t>
   </si>
   <si>
     <t>Actual Result</t>
@@ -65,25 +59,23 @@
     <t>TC_BVA_BASE</t>
   </si>
   <si>
-    <t>Order</t>
-  </si>
-  <si>
-    <t>Tất cả biến ở giá trị danh định</t>
-  </si>
-  <si>
-    <t>Nominal: (50, 500, 150000)</t>
-  </si>
-  <si>
-    <t>POST</t>
-  </si>
-  <si>
-    <t>/api/orders</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 50, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=7.500.000đ, discount=500đ, final=7.499.500đ</t>
+    <t>Tất cả biến ở giá trị danh định (Nominal BVA)</t>
+  </si>
+  <si>
+    <t>Tài khoản đã đăng nhập, điểm tích lũy &gt;= 500</t>
+  </si>
+  <si>
+    <t>1. Gửi request POST đến /api/orders
+2. Kiểm tra response trả về</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 50
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 7.500.000đ, discount = 500đ, final = 7.499.500đ</t>
   </si>
   <si>
     <t>HTTP 201 Created</t>
@@ -95,184 +87,193 @@
     <t>TC_BVA_Q_01</t>
   </si>
   <si>
-    <t>Số lượng món biên tối thiểu</t>
-  </si>
-  <si>
-    <t>quantity: Min = 1</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 1, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=150.000đ, discount=500đ, final=149.500đ</t>
+    <t>Kiểm tra số lượng món biên tối thiểu (Min = 1)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 1
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 150.000đ, discount = 500đ, final = 149.500đ</t>
   </si>
   <si>
     <t>TC_BVA_Q_02</t>
   </si>
   <si>
-    <t>Số lượng món lân cận tối thiểu</t>
-  </si>
-  <si>
-    <t>quantity: Min+ = 2</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 2, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=300.000đ, discount=500đ, final=299.500đ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HTTP 201 Created </t>
+    <t>Kiểm tra số lượng món lân cận tối thiểu (Min+ = 2)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 2
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 300.000đ, discount = 500đ, final = 299.500đ</t>
   </si>
   <si>
     <t>TC_BVA_Q_03</t>
   </si>
   <si>
-    <t>Số lượng món lân cận tối đa</t>
-  </si>
-  <si>
-    <t>quantity: Max- = 98</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 98, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=14.700.000đ, discount=500đ, final=14.699.500đ</t>
+    <t>Kiểm tra số lượng món lân cận tối đa (Max- = 98)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 98
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 14.700.000đ, discount = 500đ, final = 14.699.500đ</t>
   </si>
   <si>
     <t>TC_BVA_Q_04</t>
   </si>
   <si>
-    <t>Số lượng món biên tối đa</t>
-  </si>
-  <si>
-    <t>quantity: Max = 99</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 99, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=14.850.000đ, discount=500đ, final=14.849.500đ</t>
+    <t>Kiểm tra số lượng món biên tối đa (Max = 99)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 99
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 14.850.000đ, discount = 500đ, final = 14.849.500đ</t>
   </si>
   <si>
     <t>TC_BVA_P_01</t>
   </si>
   <si>
-    <t>Điểm tích lũy biên tối thiểu</t>
-  </si>
-  <si>
-    <t>used_points: Min = 0</t>
-  </si>
-  <si>
-    <t>used_points: 0, quantity: 50, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=7.500.000đ, discount=0đ, final=7.500.000đ</t>
+    <t>Kiểm tra điểm tích lũy biên tối thiểu (Min = 0)</t>
+  </si>
+  <si>
+    <t>Tài khoản đã đăng nhập</t>
+  </si>
+  <si>
+    <t>used_points: 0
+quantity: 50
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 7.500.000đ, discount = 0đ, final = 7.500.000đ</t>
   </si>
   <si>
     <t>TC_BVA_P_02</t>
   </si>
   <si>
-    <t>Điểm tích lũy lân cận tối thiểu</t>
-  </si>
-  <si>
-    <t>used_points: Min+ = 1</t>
-  </si>
-  <si>
-    <t>used_points: 1, quantity: 50, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=7.500.000đ, discount=1đ, final=7.499.999đ</t>
+    <t>Kiểm tra điểm tích lũy lân cận tối thiểu (Min+ = 1)</t>
+  </si>
+  <si>
+    <t>Tài khoản đã đăng nhập, điểm tích lũy &gt;= 1</t>
+  </si>
+  <si>
+    <t>used_points: 1
+quantity: 50
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 7.500.000đ, discount = 1đ, final = 7.499.999đ</t>
   </si>
   <si>
     <t>TC_BVA_P_03</t>
   </si>
   <si>
-    <t>Điểm tích lũy lân cận tối đa</t>
-  </si>
-  <si>
-    <t>used_points: Max- = 7.499.999</t>
-  </si>
-  <si>
-    <t>used_points: 7499999, quantity: 50, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=7.500.000đ, discount=7.499.999đ, final=1đ</t>
+    <t>Kiểm tra điểm tích lũy lân cận tối đa (Max- = 7.499.999)</t>
+  </si>
+  <si>
+    <t>Tài khoản đã đăng nhập, điểm tích lũy &gt;= 7.499.999</t>
+  </si>
+  <si>
+    <t>used_points: 7499999
+quantity: 50
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 7.500.000đ, discount = 7.499.999đ, final = 1đ</t>
   </si>
   <si>
     <t>TC_BVA_P_04</t>
   </si>
   <si>
-    <t>Điểm tích lũy biên tối đa</t>
-  </si>
-  <si>
-    <t>used_points: Max = 7.500.000</t>
-  </si>
-  <si>
-    <t>used_points: 7500000, quantity: 50, price: 150000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=7.500.000đ, discount=7.500.000đ, final=0đ</t>
+    <t>Kiểm tra điểm tích lũy biên tối đa (Max = 7.500.000)</t>
+  </si>
+  <si>
+    <t>Tài khoản đã đăng nhập, điểm tích lũy &gt;= 7.500.000</t>
+  </si>
+  <si>
+    <t>used_points: 7500000
+quantity: 50
+price: 150000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 7.500.000đ, discount = 7.500.000đ, final = 0đ</t>
   </si>
   <si>
     <t>TC_BVA_S_01</t>
   </si>
   <si>
-    <t>Đơn giá món biên tối thiểu</t>
-  </si>
-  <si>
-    <t>price: Min = 1.000đ</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 50, price: 1000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=50.000đ, discount=500đ, final=49.500đ</t>
+    <t>Kiểm tra đơn giá món biên tối thiểu (Min = 1.000đ)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 50
+price: 1000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 50.000đ, discount = 500đ, final = 49.500đ</t>
   </si>
   <si>
     <t>TC_BVA_S_02</t>
   </si>
   <si>
-    <t>Đơn giá món lân cận tối thiểu</t>
-  </si>
-  <si>
-    <t>price: Min+ = 2.000đ</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 50, price: 2000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=100.000đ, discount=500đ, final=99.500đ</t>
+    <t>Kiểm tra đơn giá món lân cận tối thiểu (Min+ = 2.000đ)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 50
+price: 2000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 100.000đ, discount = 500đ, final = 99.500đ</t>
   </si>
   <si>
     <t>TC_BVA_S_03</t>
   </si>
   <si>
-    <t>Đơn giá món lân cận tối đa</t>
-  </si>
-  <si>
-    <t>price: Max- = 99.999.000đ</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 50, price: 99999000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=4.999.950.000đ, discount=500đ, final=4.999.949.500đ</t>
+    <t>Kiểm tra đơn giá món lân cận tối đa (Max- = 99.999.000đ)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 50
+price: 99999000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 4.999.950.000đ, discount = 500đ, final = 4.999.949.500đ</t>
   </si>
   <si>
     <t>TC_BVA_S_04</t>
   </si>
   <si>
-    <t>Đơn giá món biên tối đa</t>
-  </si>
-  <si>
-    <t>price: Max = 100.000.000đ</t>
-  </si>
-  <si>
-    <t>used_points: 500, quantity: 50, price: 100000000</t>
-  </si>
-  <si>
-    <t>HTTP 201; total=5.000.000.000đ, discount=500đ, final=4.999.999.500đ</t>
+    <t>Kiểm tra đơn giá món biên tối đa (Max = 100.000.000đ)</t>
+  </si>
+  <si>
+    <t>used_points: 500
+quantity: 50
+price: 100000000</t>
+  </si>
+  <si>
+    <t>HTTP 201 Created;
+total = 5.000.000.000đ, discount = 500đ, final = 4.999.999.500đ</t>
   </si>
 </sst>
 </file>
@@ -321,14 +322,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF375623"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -477,7 +478,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -486,13 +487,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF004AC6"/>
+        <fgColor theme="4" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.25"/>
         <bgColor rgb="FF004AC6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
+        <fgColor theme="4" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.25"/>
         <bgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
@@ -510,7 +529,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
+        <fgColor theme="0"/>
         <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
@@ -867,7 +886,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -891,16 +910,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -909,112 +928,99 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1026,8 +1032,26 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1082,6 +1106,12 @@
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="0079F9BF"/>
+      <color rgb="00D0FFD2"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1379,757 +1409,636 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="3" max="3" width="41.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="33.1111111111111" customWidth="1"/>
+    <col min="5" max="5" width="39.7777777777778" customWidth="1"/>
+    <col min="6" max="6" width="32.1111111111111" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
-    <col min="8" max="11" width="32" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
+    <col min="12" max="12" width="12" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:12">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="1" customFormat="1" ht="30" customHeight="1" spans="1:12">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="4"/>
+      <c r="L1" s="5"/>
+    </row>
+    <row r="2" ht="42" customHeight="1" spans="1:12">
+      <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-    </row>
-    <row r="2" ht="42" customHeight="1" spans="1:12">
-      <c r="A2" s="3" t="s">
+      <c r="C2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="K2" s="8"/>
+      <c r="L2" s="10"/>
+    </row>
+    <row r="3" ht="42" customHeight="1" spans="1:12">
+      <c r="A3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="B3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="C3" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="F3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="7"/>
-      <c r="L2" s="8"/>
-    </row>
-    <row r="3" ht="42" customHeight="1" spans="1:12">
-      <c r="A3" s="9" t="s">
+      <c r="G3" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" s="13"/>
+      <c r="L3" s="10"/>
+    </row>
+    <row r="4" ht="42" customHeight="1" spans="1:12">
+      <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="11" t="s">
+      <c r="E4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="H4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="11" t="s">
+      <c r="K4" s="8"/>
+      <c r="L4" s="10"/>
+    </row>
+    <row r="5" ht="42" customHeight="1" spans="1:12">
+      <c r="A5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="7"/>
-      <c r="L3" s="8"/>
-    </row>
-    <row r="4" ht="42" customHeight="1" spans="1:12">
-      <c r="A4" s="3" t="s">
+      <c r="B5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E5" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="G5" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="H5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="K5" s="13"/>
+      <c r="L5" s="10"/>
+    </row>
+    <row r="6" ht="42" customHeight="1" spans="1:12">
+      <c r="A6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="B6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="C6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="7"/>
-      <c r="L4" s="8"/>
-    </row>
-    <row r="5" ht="42" customHeight="1" spans="1:12">
-      <c r="A5" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="G6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="10"/>
+    </row>
+    <row r="7" ht="42" customHeight="1" spans="1:12">
+      <c r="A7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="10" t="s">
+      <c r="E7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="H7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="7"/>
-      <c r="L5" s="8"/>
-    </row>
-    <row r="6" ht="42" customHeight="1" spans="1:12">
-      <c r="A6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="K7" s="13"/>
+      <c r="L7" s="10"/>
+    </row>
+    <row r="8" ht="42" customHeight="1" spans="1:12">
+      <c r="A8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="4" t="s">
+      <c r="E8" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="H8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="7"/>
-      <c r="L6" s="8"/>
-    </row>
-    <row r="7" ht="42" customHeight="1" spans="1:12">
-      <c r="A7" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="10" t="s">
+      <c r="K8" s="8"/>
+      <c r="L8" s="10"/>
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="1:12">
+      <c r="A9" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" s="10" t="s">
+      <c r="E9" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="H9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="7"/>
-      <c r="L7" s="8"/>
-    </row>
-    <row r="8" ht="42" customHeight="1" spans="1:12">
-      <c r="A8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="K9" s="13"/>
+      <c r="L9" s="10"/>
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="1:12">
+      <c r="A10" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="E10" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="H10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" s="7"/>
-      <c r="L8" s="8"/>
-    </row>
-    <row r="9" ht="42" customHeight="1" spans="1:12">
-      <c r="A9" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" s="10" t="s">
+      <c r="K10" s="8"/>
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" ht="42" customHeight="1" spans="1:12">
+      <c r="A11" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="10" t="s">
+      <c r="E11" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G11" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="H11" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="7"/>
-      <c r="L9" s="8"/>
-    </row>
-    <row r="10" ht="42" customHeight="1" spans="1:12">
-      <c r="A10" s="3" t="s">
+      <c r="K11" s="13"/>
+      <c r="L11" s="10"/>
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="1:12">
+      <c r="A12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B12" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="E12" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F12" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="H12" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="5" t="s">
+      <c r="K12" s="8"/>
+      <c r="L12" s="10"/>
+    </row>
+    <row r="13" ht="42" customHeight="1" spans="1:12">
+      <c r="A13" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="8"/>
-    </row>
-    <row r="11" ht="42" customHeight="1" spans="1:12">
-      <c r="A11" s="9" t="s">
+      <c r="B13" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C13" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="E13" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="F13" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="G13" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="H13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="K13" s="13"/>
+      <c r="L13" s="10"/>
+    </row>
+    <row r="14" ht="42" customHeight="1" spans="1:12">
+      <c r="A14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="B14" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="I11" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="8"/>
-    </row>
-    <row r="12" ht="42" customHeight="1" spans="1:12">
-      <c r="A12" s="3" t="s">
+      <c r="C14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="F14" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E12" s="4" t="s">
+      <c r="G14" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="H14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" s="7"/>
-      <c r="L12" s="8"/>
-    </row>
-    <row r="13" ht="42" customHeight="1" spans="1:12">
-      <c r="A13" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="7"/>
-      <c r="L13" s="8"/>
-    </row>
-    <row r="14" ht="42" customHeight="1" spans="1:12">
-      <c r="A14" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" s="7"/>
-      <c r="L14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="10"/>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:12">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="8"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="10"/>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:12">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="8"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="10"/>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:12">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="8"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="10"/>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:12">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="8"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="10"/>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:12">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-      <c r="L19" s="8"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="10"/>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:12">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="8"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="10"/>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:12">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="8"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="10"/>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:12">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="8"/>
+      <c r="A22" s="14"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="10"/>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:12">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="8"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="K23" s="15"/>
+      <c r="L23" s="10"/>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:12">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="8"/>
+      <c r="A24" s="14"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="10"/>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:12">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="8"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="10"/>
     </row>
     <row r="26" ht="42" customHeight="1" spans="1:12">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="8"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="10"/>
     </row>
     <row r="27" ht="42" customHeight="1" spans="1:12">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="8"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="10"/>
     </row>
     <row r="28" ht="42" customHeight="1" spans="1:12">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="8"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="10"/>
     </row>
     <row r="29" ht="42" customHeight="1" spans="1:12">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="8"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="10"/>
     </row>
     <row r="30" ht="42" customHeight="1" spans="1:12">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="8"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="K30" s="15"/>
+      <c r="L30" s="10"/>
     </row>
     <row r="31" ht="42" customHeight="1" spans="1:12">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="8"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="10"/>
     </row>
     <row r="32" ht="42" customHeight="1" spans="1:12">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="8"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="10"/>
     </row>
     <row r="33" ht="42" customHeight="1" spans="1:12">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="8"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="10"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L33" etc:filterBottomFollowUsedRange="0">

</xml_diff>